<commit_message>
Update 6000 web data 1.0.1
</commit_message>
<xml_diff>
--- a/data_6000.xlsx
+++ b/data_6000.xlsx
@@ -5,15 +5,33 @@
     <workbookView xWindow="0" yWindow="40" windowWidth="15960" windowHeight="18080"/>
   </bookViews>
   <sheets>
-    <sheet name="แผ่นงานที่ 1" sheetId="1" r:id="rId4"/>
+    <sheet name="Machines" sheetId="1" r:id="rId4"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="1">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="7">
   <si>
-    <t>ตาราง 1</t>
+    <t>ID Machine</t>
+  </si>
+  <si>
+    <t>Model</t>
+  </si>
+  <si>
+    <t>No.</t>
+  </si>
+  <si>
+    <t>Department</t>
+  </si>
+  <si>
+    <t>Test</t>
+  </si>
+  <si>
+    <t>Test 6000</t>
+  </si>
+  <si>
+    <t>#00</t>
   </si>
 </sst>
 </file>
@@ -23,11 +41,11 @@
   <numFmts count="1">
     <numFmt numFmtId="0" formatCode="General"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="4">
     <font>
-      <sz val="10"/>
+      <sz val="11"/>
       <color indexed="8"/>
-      <name val="Helvetica Neue"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <sz val="12"/>
@@ -35,10 +53,15 @@
       <name val="Helvetica Neue"/>
     </font>
     <font>
+      <sz val="15"/>
+      <color indexed="8"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
       <b val="1"/>
-      <sz val="10"/>
+      <sz val="11"/>
       <color indexed="8"/>
-      <name val="Helvetica Neue"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="4">
@@ -56,12 +79,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor indexed="12"/>
+        <fgColor indexed="11"/>
         <bgColor auto="1"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="8">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -71,97 +94,22 @@
     </border>
     <border>
       <left style="thin">
-        <color indexed="10"/>
+        <color indexed="8"/>
       </left>
       <right style="thin">
-        <color indexed="10"/>
+        <color indexed="8"/>
       </right>
       <top style="thin">
-        <color indexed="10"/>
+        <color indexed="8"/>
       </top>
       <bottom style="thin">
-        <color indexed="11"/>
+        <color indexed="8"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color indexed="10"/>
-      </left>
-      <right style="thin">
-        <color indexed="11"/>
-      </right>
-      <top style="thin">
-        <color indexed="11"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="10"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="11"/>
-      </left>
-      <right style="thin">
-        <color indexed="10"/>
-      </right>
-      <top style="thin">
-        <color indexed="11"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="10"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="10"/>
-      </left>
-      <right style="thin">
-        <color indexed="10"/>
-      </right>
-      <top style="thin">
-        <color indexed="11"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="10"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="10"/>
-      </left>
-      <right style="thin">
-        <color indexed="11"/>
-      </right>
-      <top style="thin">
-        <color indexed="10"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="10"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="11"/>
-      </left>
-      <right style="thin">
-        <color indexed="10"/>
-      </right>
-      <top style="thin">
-        <color indexed="10"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="10"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="10"/>
+        <color indexed="8"/>
       </left>
       <right style="thin">
         <color indexed="10"/>
@@ -177,39 +125,33 @@
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment vertical="bottom"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="1" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" borderId="2" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" borderId="3" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" borderId="4" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" borderId="6" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" borderId="7" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -228,19 +170,18 @@
       <rgbColor rgb="ffff00ff"/>
       <rgbColor rgb="ff00ffff"/>
       <rgbColor rgb="ff000000"/>
-      <rgbColor rgb="ffbdc0bf"/>
-      <rgbColor rgb="ffa5a5a5"/>
-      <rgbColor rgb="ff3f3f3f"/>
-      <rgbColor rgb="ffdbdbdb"/>
+      <rgbColor rgb="ffd3d3d3"/>
+      <rgbColor rgb="ffaaaaaa"/>
+      <rgbColor rgb="ffffffff"/>
     </indexedColors>
   </colors>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Blank">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Blank">
+    <a:clrScheme name="Office Theme">
       <a:dk1>
         <a:srgbClr val="000000"/>
       </a:dk1>
@@ -248,28 +189,28 @@
         <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="5E5E5E"/>
+        <a:srgbClr val="A7A7A7"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="D5D5D5"/>
+        <a:srgbClr val="535353"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="00A2FF"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="16E7CF"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="61D836"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="FFD932"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="FF644E"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="FF42A1"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
         <a:srgbClr val="0000FF"/>
@@ -278,7 +219,7 @@
         <a:srgbClr val="FF00FF"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Blank">
+    <a:fontScheme name="Office Theme">
       <a:majorFont>
         <a:latin typeface="Helvetica Neue"/>
         <a:ea typeface="Helvetica Neue"/>
@@ -290,7 +231,7 @@
         <a:cs typeface="Helvetica Neue"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Blank">
+    <a:fmtScheme name="Office Theme">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -363,13 +304,31 @@
       </a:lnStyleLst>
       <a:effectStyleLst>
         <a:effectStyle>
-          <a:effectLst/>
+          <a:effectLst>
+            <a:outerShdw sx="100000" sy="100000" kx="0" ky="0" algn="b" rotWithShape="0" blurRad="38100" dist="23000" dir="5400000">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
         </a:effectStyle>
         <a:effectStyle>
-          <a:effectLst/>
+          <a:effectLst>
+            <a:outerShdw sx="100000" sy="100000" kx="0" ky="0" algn="b" rotWithShape="0" blurRad="38100" dist="23000" dir="5400000">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
         </a:effectStyle>
         <a:effectStyle>
-          <a:effectLst/>
+          <a:effectLst>
+            <a:outerShdw sx="100000" sy="100000" kx="0" ky="0" algn="b" rotWithShape="0" blurRad="38100" dist="20000" dir="5400000">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
@@ -428,20 +387,29 @@
     <a:spDef>
       <a:spPr>
         <a:solidFill>
-          <a:srgbClr val="000000"/>
+          <a:srgbClr val="FFFFFF"/>
         </a:solidFill>
-        <a:ln w="12700" cap="flat">
-          <a:noFill/>
-          <a:miter lim="400000"/>
+        <a:ln w="25400" cap="flat">
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:round/>
         </a:ln>
-        <a:effectLst/>
+        <a:effectLst>
+          <a:outerShdw sx="100000" sy="100000" kx="0" ky="0" algn="b" rotWithShape="0" blurRad="38100" dist="23000" dir="5400000">
+            <a:srgbClr val="000000">
+              <a:alpha val="35000"/>
+            </a:srgbClr>
+          </a:outerShdw>
+        </a:effectLst>
         <a:sp3d/>
       </a:spPr>
-      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="50800" tIns="50800" rIns="50800" bIns="50800" numCol="1" spcCol="38100" rtlCol="0" anchor="ctr" upright="0">
+      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="45719" tIns="45719" rIns="45719" bIns="45719" numCol="1" spcCol="38100" rtlCol="0" anchor="ctr" upright="0">
         <a:spAutoFit/>
       </a:bodyPr>
       <a:lstStyle>
-        <a:defPPr marL="0" marR="0" indent="0" algn="ctr" defTabSz="584200" rtl="0" fontAlgn="auto" latinLnBrk="0" hangingPunct="0">
+        <a:defPPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="0" hangingPunct="0">
           <a:lnSpc>
             <a:spcPct val="100000"/>
           </a:lnSpc>
@@ -455,19 +423,19 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1200" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1100" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
             <a:solidFill>
-              <a:srgbClr val="FFFFFF"/>
+              <a:srgbClr val="000000"/>
             </a:solidFill>
             <a:effectLst/>
             <a:uFillTx/>
-            <a:latin typeface="Helvetica Neue Medium"/>
-            <a:ea typeface="Helvetica Neue Medium"/>
-            <a:cs typeface="Helvetica Neue Medium"/>
-            <a:sym typeface="Helvetica Neue Medium"/>
+            <a:latin typeface="Calibri"/>
+            <a:ea typeface="Calibri"/>
+            <a:cs typeface="Calibri"/>
+            <a:sym typeface="Calibri"/>
           </a:defRPr>
         </a:defPPr>
         <a:lvl1pPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="1" hangingPunct="0">
@@ -706,14 +674,20 @@
     <a:lnDef>
       <a:spPr>
         <a:noFill/>
-        <a:ln w="12700" cap="flat">
+        <a:ln w="25400" cap="flat">
           <a:solidFill>
-            <a:srgbClr val="000000"/>
+            <a:schemeClr val="accent1"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="400000"/>
+          <a:round/>
         </a:ln>
-        <a:effectLst/>
+        <a:effectLst>
+          <a:outerShdw sx="100000" sy="100000" kx="0" ky="0" algn="b" rotWithShape="0" blurRad="38100" dist="20000" dir="5400000">
+            <a:srgbClr val="000000">
+              <a:alpha val="38000"/>
+            </a:srgbClr>
+          </a:outerShdw>
+        </a:effectLst>
         <a:sp3d/>
       </a:spPr>
       <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="91439" tIns="45719" rIns="91439" bIns="45719" numCol="1" spcCol="38100" rtlCol="0" anchor="t" upright="0">
@@ -988,11 +962,11 @@
         <a:effectLst/>
         <a:sp3d/>
       </a:spPr>
-      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="50800" tIns="50800" rIns="50800" bIns="50800" numCol="1" spcCol="38100" rtlCol="0" anchor="t" upright="0">
+      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="45719" tIns="45719" rIns="45719" bIns="45719" numCol="1" spcCol="38100" rtlCol="0" anchor="t" upright="0">
         <a:spAutoFit/>
       </a:bodyPr>
       <a:lstStyle>
-        <a:defPPr marL="0" marR="0" indent="0" algn="l" defTabSz="457200" rtl="0" fontAlgn="auto" latinLnBrk="0" hangingPunct="0">
+        <a:defPPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="0" hangingPunct="0">
           <a:lnSpc>
             <a:spcPct val="100000"/>
           </a:lnSpc>
@@ -1015,10 +989,10 @@
             </a:solidFill>
             <a:effectLst/>
             <a:uFillTx/>
-            <a:latin typeface="+mn-lt"/>
-            <a:ea typeface="+mn-ea"/>
-            <a:cs typeface="+mn-cs"/>
-            <a:sym typeface="Helvetica Neue"/>
+            <a:latin typeface="Calibri"/>
+            <a:ea typeface="Calibri"/>
+            <a:cs typeface="Calibri"/>
+            <a:sym typeface="Calibri"/>
           </a:defRPr>
         </a:defPPr>
         <a:lvl1pPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="1" hangingPunct="0">
@@ -1260,228 +1234,1705 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A2:G23"/>
-  <sheetFormatPr defaultColWidth="16.3333" defaultRowHeight="19.9" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:E238"/>
+  <sheetFormatPr defaultColWidth="8" defaultRowHeight="12.75" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="7" width="16.3516" style="1" customWidth="1"/>
-    <col min="8" max="16384" width="16.3516" style="1" customWidth="1"/>
+    <col min="1" max="1" width="23.5" style="1" customWidth="1"/>
+    <col min="2" max="2" width="19.5" style="1" customWidth="1"/>
+    <col min="3" max="3" width="11.5" style="1" customWidth="1"/>
+    <col min="4" max="4" width="23.5" style="1" customWidth="1"/>
+    <col min="5" max="5" width="8" style="1" customWidth="1"/>
+    <col min="6" max="16384" width="8" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30.15" customHeight="1">
+    <row r="1" ht="12.75" customHeight="1">
       <c r="A1" t="s" s="2">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-    </row>
-    <row r="2" ht="20.25" customHeight="1">
-      <c r="A2" s="3"/>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
+      <c r="B1" t="s" s="2">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s" s="2">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s" s="2">
+        <v>3</v>
+      </c>
+      <c r="E1" s="3"/>
+    </row>
+    <row r="2" ht="12.75" customHeight="1">
+      <c r="A2" t="s" s="4">
+        <v>4</v>
+      </c>
+      <c r="B2" t="s" s="4">
+        <v>5</v>
+      </c>
+      <c r="C2" t="s" s="5">
+        <v>6</v>
+      </c>
+      <c r="D2" t="s" s="4">
+        <v>4</v>
+      </c>
       <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
-    </row>
-    <row r="3" ht="20.25" customHeight="1">
-      <c r="A3" s="4"/>
-      <c r="B3" s="5"/>
-      <c r="C3" s="6"/>
+    </row>
+    <row r="3" ht="12.75" customHeight="1">
+      <c r="A3" s="6"/>
+      <c r="B3" s="6"/>
+      <c r="C3" s="7"/>
       <c r="D3" s="6"/>
-      <c r="E3" s="6"/>
-      <c r="F3" s="6"/>
-      <c r="G3" s="6"/>
-    </row>
-    <row r="4" ht="20.05" customHeight="1">
-      <c r="A4" s="7"/>
-      <c r="B4" s="8"/>
-      <c r="C4" s="9"/>
-      <c r="D4" s="9"/>
-      <c r="E4" s="9"/>
-      <c r="F4" s="9"/>
-      <c r="G4" s="9"/>
-    </row>
-    <row r="5" ht="20.05" customHeight="1">
-      <c r="A5" s="7"/>
-      <c r="B5" s="8"/>
-      <c r="C5" s="9"/>
-      <c r="D5" s="9"/>
-      <c r="E5" s="9"/>
-      <c r="F5" s="9"/>
-      <c r="G5" s="9"/>
-    </row>
-    <row r="6" ht="20.05" customHeight="1">
-      <c r="A6" s="7"/>
-      <c r="B6" s="8"/>
-      <c r="C6" s="9"/>
-      <c r="D6" s="9"/>
-      <c r="E6" s="9"/>
-      <c r="F6" s="9"/>
-      <c r="G6" s="9"/>
-    </row>
-    <row r="7" ht="20.05" customHeight="1">
-      <c r="A7" s="7"/>
-      <c r="B7" s="8"/>
-      <c r="C7" s="9"/>
-      <c r="D7" s="9"/>
-      <c r="E7" s="9"/>
-      <c r="F7" s="9"/>
-      <c r="G7" s="9"/>
-    </row>
-    <row r="8" ht="20.05" customHeight="1">
-      <c r="A8" s="7"/>
-      <c r="B8" s="8"/>
-      <c r="C8" s="9"/>
-      <c r="D8" s="9"/>
-      <c r="E8" s="9"/>
-      <c r="F8" s="9"/>
-      <c r="G8" s="9"/>
-    </row>
-    <row r="9" ht="20.05" customHeight="1">
-      <c r="A9" s="7"/>
-      <c r="B9" s="8"/>
-      <c r="C9" s="9"/>
-      <c r="D9" s="9"/>
-      <c r="E9" s="9"/>
-      <c r="F9" s="9"/>
-      <c r="G9" s="9"/>
-    </row>
-    <row r="10" ht="20.05" customHeight="1">
-      <c r="A10" s="7"/>
-      <c r="B10" s="8"/>
-      <c r="C10" s="9"/>
-      <c r="D10" s="9"/>
-      <c r="E10" s="9"/>
-      <c r="F10" s="9"/>
-      <c r="G10" s="9"/>
-    </row>
-    <row r="11" ht="20.05" customHeight="1">
-      <c r="A11" s="7"/>
-      <c r="B11" s="8"/>
-      <c r="C11" s="9"/>
-      <c r="D11" s="9"/>
-      <c r="E11" s="9"/>
-      <c r="F11" s="9"/>
-      <c r="G11" s="9"/>
-    </row>
-    <row r="12" ht="20.05" customHeight="1">
-      <c r="A12" s="7"/>
-      <c r="B12" s="8"/>
-      <c r="C12" s="9"/>
-      <c r="D12" s="9"/>
-      <c r="E12" s="9"/>
-      <c r="F12" s="9"/>
-      <c r="G12" s="9"/>
-    </row>
-    <row r="13" ht="20.05" customHeight="1">
-      <c r="A13" s="7"/>
-      <c r="B13" s="8"/>
-      <c r="C13" s="9"/>
-      <c r="D13" s="9"/>
-      <c r="E13" s="9"/>
-      <c r="F13" s="9"/>
-      <c r="G13" s="9"/>
-    </row>
-    <row r="14" ht="20.05" customHeight="1">
-      <c r="A14" s="7"/>
-      <c r="B14" s="8"/>
-      <c r="C14" s="9"/>
-      <c r="D14" s="9"/>
-      <c r="E14" s="9"/>
-      <c r="F14" s="9"/>
-      <c r="G14" s="9"/>
-    </row>
-    <row r="15" ht="20.05" customHeight="1">
-      <c r="A15" s="7"/>
-      <c r="B15" s="8"/>
-      <c r="C15" s="9"/>
-      <c r="D15" s="9"/>
-      <c r="E15" s="9"/>
-      <c r="F15" s="9"/>
-      <c r="G15" s="9"/>
-    </row>
-    <row r="16" ht="20.05" customHeight="1">
-      <c r="A16" s="7"/>
-      <c r="B16" s="8"/>
-      <c r="C16" s="9"/>
-      <c r="D16" s="9"/>
-      <c r="E16" s="9"/>
-      <c r="F16" s="9"/>
-      <c r="G16" s="9"/>
-    </row>
-    <row r="17" ht="20.05" customHeight="1">
-      <c r="A17" s="7"/>
-      <c r="B17" s="8"/>
-      <c r="C17" s="9"/>
-      <c r="D17" s="9"/>
-      <c r="E17" s="9"/>
-      <c r="F17" s="9"/>
-      <c r="G17" s="9"/>
-    </row>
-    <row r="18" ht="20.05" customHeight="1">
-      <c r="A18" s="7"/>
-      <c r="B18" s="8"/>
-      <c r="C18" s="9"/>
-      <c r="D18" s="9"/>
-      <c r="E18" s="9"/>
-      <c r="F18" s="9"/>
-      <c r="G18" s="9"/>
-    </row>
-    <row r="19" ht="20.05" customHeight="1">
-      <c r="A19" s="7"/>
-      <c r="B19" s="8"/>
-      <c r="C19" s="9"/>
-      <c r="D19" s="9"/>
-      <c r="E19" s="9"/>
-      <c r="F19" s="9"/>
-      <c r="G19" s="9"/>
-    </row>
-    <row r="20" ht="20.05" customHeight="1">
-      <c r="A20" s="7"/>
-      <c r="B20" s="8"/>
-      <c r="C20" s="9"/>
-      <c r="D20" s="9"/>
-      <c r="E20" s="9"/>
-      <c r="F20" s="9"/>
-      <c r="G20" s="9"/>
-    </row>
-    <row r="21" ht="20.05" customHeight="1">
-      <c r="A21" s="7"/>
-      <c r="B21" s="8"/>
-      <c r="C21" s="9"/>
-      <c r="D21" s="9"/>
-      <c r="E21" s="9"/>
-      <c r="F21" s="9"/>
-      <c r="G21" s="9"/>
-    </row>
-    <row r="22" ht="20.05" customHeight="1">
-      <c r="A22" s="7"/>
-      <c r="B22" s="8"/>
-      <c r="C22" s="9"/>
-      <c r="D22" s="9"/>
-      <c r="E22" s="9"/>
-      <c r="F22" s="9"/>
-      <c r="G22" s="9"/>
-    </row>
-    <row r="23" ht="20.05" customHeight="1">
-      <c r="A23" s="7"/>
-      <c r="B23" s="8"/>
-      <c r="C23" s="9"/>
-      <c r="D23" s="9"/>
-      <c r="E23" s="9"/>
-      <c r="F23" s="9"/>
-      <c r="G23" s="9"/>
+      <c r="E3" s="3"/>
+    </row>
+    <row r="4" ht="12.75" customHeight="1">
+      <c r="A4" s="6"/>
+      <c r="B4" s="6"/>
+      <c r="C4" s="7"/>
+      <c r="D4" s="6"/>
+      <c r="E4" s="3"/>
+    </row>
+    <row r="5" ht="12.75" customHeight="1">
+      <c r="A5" s="6"/>
+      <c r="B5" s="6"/>
+      <c r="C5" s="7"/>
+      <c r="D5" s="6"/>
+      <c r="E5" s="3"/>
+    </row>
+    <row r="6" ht="12.75" customHeight="1">
+      <c r="A6" s="6"/>
+      <c r="B6" s="6"/>
+      <c r="C6" s="7"/>
+      <c r="D6" s="6"/>
+      <c r="E6" s="3"/>
+    </row>
+    <row r="7" ht="12.75" customHeight="1">
+      <c r="A7" s="6"/>
+      <c r="B7" s="6"/>
+      <c r="C7" s="7"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="3"/>
+    </row>
+    <row r="8" ht="12.75" customHeight="1">
+      <c r="A8" s="6"/>
+      <c r="B8" s="6"/>
+      <c r="C8" s="7"/>
+      <c r="D8" s="6"/>
+      <c r="E8" s="3"/>
+    </row>
+    <row r="9" ht="12.75" customHeight="1">
+      <c r="A9" s="6"/>
+      <c r="B9" s="6"/>
+      <c r="C9" s="7"/>
+      <c r="D9" s="6"/>
+      <c r="E9" s="3"/>
+    </row>
+    <row r="10" ht="12.75" customHeight="1">
+      <c r="A10" s="6"/>
+      <c r="B10" s="6"/>
+      <c r="C10" s="7"/>
+      <c r="D10" s="6"/>
+      <c r="E10" s="3"/>
+    </row>
+    <row r="11" ht="12.75" customHeight="1">
+      <c r="A11" s="6"/>
+      <c r="B11" s="6"/>
+      <c r="C11" s="7"/>
+      <c r="D11" s="6"/>
+      <c r="E11" s="3"/>
+    </row>
+    <row r="12" ht="12.75" customHeight="1">
+      <c r="A12" s="6"/>
+      <c r="B12" s="6"/>
+      <c r="C12" s="7"/>
+      <c r="D12" s="6"/>
+      <c r="E12" s="3"/>
+    </row>
+    <row r="13" ht="12.75" customHeight="1">
+      <c r="A13" s="6"/>
+      <c r="B13" s="6"/>
+      <c r="C13" s="7"/>
+      <c r="D13" s="6"/>
+      <c r="E13" s="3"/>
+    </row>
+    <row r="14" ht="12.75" customHeight="1">
+      <c r="A14" s="6"/>
+      <c r="B14" s="6"/>
+      <c r="C14" s="7"/>
+      <c r="D14" s="6"/>
+      <c r="E14" s="3"/>
+    </row>
+    <row r="15" ht="12.75" customHeight="1">
+      <c r="A15" s="6"/>
+      <c r="B15" s="6"/>
+      <c r="C15" s="7"/>
+      <c r="D15" s="6"/>
+      <c r="E15" s="3"/>
+    </row>
+    <row r="16" ht="12.75" customHeight="1">
+      <c r="A16" s="6"/>
+      <c r="B16" s="6"/>
+      <c r="C16" s="7"/>
+      <c r="D16" s="6"/>
+      <c r="E16" s="3"/>
+    </row>
+    <row r="17" ht="12.75" customHeight="1">
+      <c r="A17" s="6"/>
+      <c r="B17" s="6"/>
+      <c r="C17" s="7"/>
+      <c r="D17" s="6"/>
+      <c r="E17" s="3"/>
+    </row>
+    <row r="18" ht="12.75" customHeight="1">
+      <c r="A18" s="6"/>
+      <c r="B18" s="6"/>
+      <c r="C18" s="7"/>
+      <c r="D18" s="6"/>
+      <c r="E18" s="3"/>
+    </row>
+    <row r="19" ht="12.75" customHeight="1">
+      <c r="A19" s="6"/>
+      <c r="B19" s="6"/>
+      <c r="C19" s="7"/>
+      <c r="D19" s="6"/>
+      <c r="E19" s="3"/>
+    </row>
+    <row r="20" ht="12.75" customHeight="1">
+      <c r="A20" s="6"/>
+      <c r="B20" s="6"/>
+      <c r="C20" s="7"/>
+      <c r="D20" s="6"/>
+      <c r="E20" s="3"/>
+    </row>
+    <row r="21" ht="12.75" customHeight="1">
+      <c r="A21" s="6"/>
+      <c r="B21" s="6"/>
+      <c r="C21" s="7"/>
+      <c r="D21" s="6"/>
+      <c r="E21" s="3"/>
+    </row>
+    <row r="22" ht="12.75" customHeight="1">
+      <c r="A22" s="6"/>
+      <c r="B22" s="6"/>
+      <c r="C22" s="7"/>
+      <c r="D22" s="6"/>
+      <c r="E22" s="3"/>
+    </row>
+    <row r="23" ht="12.75" customHeight="1">
+      <c r="A23" s="6"/>
+      <c r="B23" s="6"/>
+      <c r="C23" s="7"/>
+      <c r="D23" s="6"/>
+      <c r="E23" s="3"/>
+    </row>
+    <row r="24" ht="12.75" customHeight="1">
+      <c r="A24" s="6"/>
+      <c r="B24" s="6"/>
+      <c r="C24" s="7"/>
+      <c r="D24" s="6"/>
+      <c r="E24" s="3"/>
+    </row>
+    <row r="25" ht="12.75" customHeight="1">
+      <c r="A25" s="6"/>
+      <c r="B25" s="6"/>
+      <c r="C25" s="7"/>
+      <c r="D25" s="6"/>
+      <c r="E25" s="3"/>
+    </row>
+    <row r="26" ht="12.75" customHeight="1">
+      <c r="A26" s="6"/>
+      <c r="B26" s="6"/>
+      <c r="C26" s="7"/>
+      <c r="D26" s="6"/>
+      <c r="E26" s="3"/>
+    </row>
+    <row r="27" ht="12.75" customHeight="1">
+      <c r="A27" s="6"/>
+      <c r="B27" s="6"/>
+      <c r="C27" s="7"/>
+      <c r="D27" s="6"/>
+      <c r="E27" s="3"/>
+    </row>
+    <row r="28" ht="12.75" customHeight="1">
+      <c r="A28" s="6"/>
+      <c r="B28" s="6"/>
+      <c r="C28" s="7"/>
+      <c r="D28" s="6"/>
+      <c r="E28" s="3"/>
+    </row>
+    <row r="29" ht="12.75" customHeight="1">
+      <c r="A29" s="6"/>
+      <c r="B29" s="6"/>
+      <c r="C29" s="7"/>
+      <c r="D29" s="6"/>
+      <c r="E29" s="3"/>
+    </row>
+    <row r="30" ht="12.75" customHeight="1">
+      <c r="A30" s="6"/>
+      <c r="B30" s="6"/>
+      <c r="C30" s="7"/>
+      <c r="D30" s="6"/>
+      <c r="E30" s="3"/>
+    </row>
+    <row r="31" ht="12.75" customHeight="1">
+      <c r="A31" s="6"/>
+      <c r="B31" s="6"/>
+      <c r="C31" s="7"/>
+      <c r="D31" s="6"/>
+      <c r="E31" s="3"/>
+    </row>
+    <row r="32" ht="12.75" customHeight="1">
+      <c r="A32" s="6"/>
+      <c r="B32" s="6"/>
+      <c r="C32" s="7"/>
+      <c r="D32" s="6"/>
+      <c r="E32" s="3"/>
+    </row>
+    <row r="33" ht="12.75" customHeight="1">
+      <c r="A33" s="6"/>
+      <c r="B33" s="6"/>
+      <c r="C33" s="7"/>
+      <c r="D33" s="6"/>
+      <c r="E33" s="3"/>
+    </row>
+    <row r="34" ht="12.75" customHeight="1">
+      <c r="A34" s="6"/>
+      <c r="B34" s="6"/>
+      <c r="C34" s="7"/>
+      <c r="D34" s="6"/>
+      <c r="E34" s="3"/>
+    </row>
+    <row r="35" ht="12.75" customHeight="1">
+      <c r="A35" s="6"/>
+      <c r="B35" s="6"/>
+      <c r="C35" s="7"/>
+      <c r="D35" s="6"/>
+      <c r="E35" s="3"/>
+    </row>
+    <row r="36" ht="12.75" customHeight="1">
+      <c r="A36" s="6"/>
+      <c r="B36" s="6"/>
+      <c r="C36" s="7"/>
+      <c r="D36" s="6"/>
+      <c r="E36" s="3"/>
+    </row>
+    <row r="37" ht="12.75" customHeight="1">
+      <c r="A37" s="6"/>
+      <c r="B37" s="6"/>
+      <c r="C37" s="7"/>
+      <c r="D37" s="6"/>
+      <c r="E37" s="3"/>
+    </row>
+    <row r="38" ht="12.75" customHeight="1">
+      <c r="A38" s="6"/>
+      <c r="B38" s="6"/>
+      <c r="C38" s="7"/>
+      <c r="D38" s="6"/>
+      <c r="E38" s="3"/>
+    </row>
+    <row r="39" ht="12.75" customHeight="1">
+      <c r="A39" s="6"/>
+      <c r="B39" s="6"/>
+      <c r="C39" s="7"/>
+      <c r="D39" s="6"/>
+      <c r="E39" s="3"/>
+    </row>
+    <row r="40" ht="12.75" customHeight="1">
+      <c r="A40" s="6"/>
+      <c r="B40" s="6"/>
+      <c r="C40" s="7"/>
+      <c r="D40" s="6"/>
+      <c r="E40" s="3"/>
+    </row>
+    <row r="41" ht="12.75" customHeight="1">
+      <c r="A41" s="6"/>
+      <c r="B41" s="6"/>
+      <c r="C41" s="7"/>
+      <c r="D41" s="6"/>
+      <c r="E41" s="3"/>
+    </row>
+    <row r="42" ht="12.75" customHeight="1">
+      <c r="A42" s="6"/>
+      <c r="B42" s="6"/>
+      <c r="C42" s="7"/>
+      <c r="D42" s="6"/>
+      <c r="E42" s="3"/>
+    </row>
+    <row r="43" ht="12.75" customHeight="1">
+      <c r="A43" s="6"/>
+      <c r="B43" s="6"/>
+      <c r="C43" s="7"/>
+      <c r="D43" s="6"/>
+      <c r="E43" s="3"/>
+    </row>
+    <row r="44" ht="12.75" customHeight="1">
+      <c r="A44" s="6"/>
+      <c r="B44" s="6"/>
+      <c r="C44" s="7"/>
+      <c r="D44" s="6"/>
+      <c r="E44" s="3"/>
+    </row>
+    <row r="45" ht="12.75" customHeight="1">
+      <c r="A45" s="6"/>
+      <c r="B45" s="6"/>
+      <c r="C45" s="7"/>
+      <c r="D45" s="6"/>
+      <c r="E45" s="3"/>
+    </row>
+    <row r="46" ht="12.75" customHeight="1">
+      <c r="A46" s="6"/>
+      <c r="B46" s="6"/>
+      <c r="C46" s="7"/>
+      <c r="D46" s="6"/>
+      <c r="E46" s="3"/>
+    </row>
+    <row r="47" ht="12.75" customHeight="1">
+      <c r="A47" s="6"/>
+      <c r="B47" s="6"/>
+      <c r="C47" s="7"/>
+      <c r="D47" s="6"/>
+      <c r="E47" s="3"/>
+    </row>
+    <row r="48" ht="12.75" customHeight="1">
+      <c r="A48" s="6"/>
+      <c r="B48" s="6"/>
+      <c r="C48" s="7"/>
+      <c r="D48" s="6"/>
+      <c r="E48" s="3"/>
+    </row>
+    <row r="49" ht="12.75" customHeight="1">
+      <c r="A49" s="6"/>
+      <c r="B49" s="6"/>
+      <c r="C49" s="7"/>
+      <c r="D49" s="6"/>
+      <c r="E49" s="3"/>
+    </row>
+    <row r="50" ht="12.75" customHeight="1">
+      <c r="A50" s="6"/>
+      <c r="B50" s="6"/>
+      <c r="C50" s="7"/>
+      <c r="D50" s="6"/>
+      <c r="E50" s="3"/>
+    </row>
+    <row r="51" ht="12.75" customHeight="1">
+      <c r="A51" s="6"/>
+      <c r="B51" s="6"/>
+      <c r="C51" s="7"/>
+      <c r="D51" s="6"/>
+      <c r="E51" s="3"/>
+    </row>
+    <row r="52" ht="12.75" customHeight="1">
+      <c r="A52" s="6"/>
+      <c r="B52" s="6"/>
+      <c r="C52" s="7"/>
+      <c r="D52" s="6"/>
+      <c r="E52" s="3"/>
+    </row>
+    <row r="53" ht="12.75" customHeight="1">
+      <c r="A53" s="6"/>
+      <c r="B53" s="6"/>
+      <c r="C53" s="7"/>
+      <c r="D53" s="6"/>
+      <c r="E53" s="3"/>
+    </row>
+    <row r="54" ht="12.75" customHeight="1">
+      <c r="A54" s="6"/>
+      <c r="B54" s="6"/>
+      <c r="C54" s="7"/>
+      <c r="D54" s="6"/>
+      <c r="E54" s="3"/>
+    </row>
+    <row r="55" ht="12.75" customHeight="1">
+      <c r="A55" s="6"/>
+      <c r="B55" s="6"/>
+      <c r="C55" s="7"/>
+      <c r="D55" s="6"/>
+      <c r="E55" s="3"/>
+    </row>
+    <row r="56" ht="12.75" customHeight="1">
+      <c r="A56" s="6"/>
+      <c r="B56" s="6"/>
+      <c r="C56" s="7"/>
+      <c r="D56" s="6"/>
+      <c r="E56" s="3"/>
+    </row>
+    <row r="57" ht="12.75" customHeight="1">
+      <c r="A57" s="6"/>
+      <c r="B57" s="6"/>
+      <c r="C57" s="7"/>
+      <c r="D57" s="6"/>
+      <c r="E57" s="3"/>
+    </row>
+    <row r="58" ht="12.75" customHeight="1">
+      <c r="A58" s="6"/>
+      <c r="B58" s="6"/>
+      <c r="C58" s="7"/>
+      <c r="D58" s="6"/>
+      <c r="E58" s="3"/>
+    </row>
+    <row r="59" ht="12.75" customHeight="1">
+      <c r="A59" s="6"/>
+      <c r="B59" s="6"/>
+      <c r="C59" s="7"/>
+      <c r="D59" s="6"/>
+      <c r="E59" s="3"/>
+    </row>
+    <row r="60" ht="12.75" customHeight="1">
+      <c r="A60" s="6"/>
+      <c r="B60" s="6"/>
+      <c r="C60" s="7"/>
+      <c r="D60" s="6"/>
+      <c r="E60" s="3"/>
+    </row>
+    <row r="61" ht="12.75" customHeight="1">
+      <c r="A61" s="6"/>
+      <c r="B61" s="6"/>
+      <c r="C61" s="7"/>
+      <c r="D61" s="6"/>
+      <c r="E61" s="3"/>
+    </row>
+    <row r="62" ht="12.75" customHeight="1">
+      <c r="A62" s="6"/>
+      <c r="B62" s="6"/>
+      <c r="C62" s="7"/>
+      <c r="D62" s="6"/>
+      <c r="E62" s="3"/>
+    </row>
+    <row r="63" ht="12.75" customHeight="1">
+      <c r="A63" s="6"/>
+      <c r="B63" s="6"/>
+      <c r="C63" s="7"/>
+      <c r="D63" s="6"/>
+      <c r="E63" s="3"/>
+    </row>
+    <row r="64" ht="12.75" customHeight="1">
+      <c r="A64" s="6"/>
+      <c r="B64" s="6"/>
+      <c r="C64" s="7"/>
+      <c r="D64" s="6"/>
+      <c r="E64" s="3"/>
+    </row>
+    <row r="65" ht="12.75" customHeight="1">
+      <c r="A65" s="6"/>
+      <c r="B65" s="6"/>
+      <c r="C65" s="7"/>
+      <c r="D65" s="6"/>
+      <c r="E65" s="3"/>
+    </row>
+    <row r="66" ht="12.75" customHeight="1">
+      <c r="A66" s="6"/>
+      <c r="B66" s="6"/>
+      <c r="C66" s="7"/>
+      <c r="D66" s="6"/>
+      <c r="E66" s="3"/>
+    </row>
+    <row r="67" ht="12.75" customHeight="1">
+      <c r="A67" s="6"/>
+      <c r="B67" s="6"/>
+      <c r="C67" s="7"/>
+      <c r="D67" s="6"/>
+      <c r="E67" s="3"/>
+    </row>
+    <row r="68" ht="12.75" customHeight="1">
+      <c r="A68" s="6"/>
+      <c r="B68" s="6"/>
+      <c r="C68" s="7"/>
+      <c r="D68" s="6"/>
+      <c r="E68" s="3"/>
+    </row>
+    <row r="69" ht="12.75" customHeight="1">
+      <c r="A69" s="6"/>
+      <c r="B69" s="6"/>
+      <c r="C69" s="7"/>
+      <c r="D69" s="6"/>
+      <c r="E69" s="3"/>
+    </row>
+    <row r="70" ht="12.75" customHeight="1">
+      <c r="A70" s="6"/>
+      <c r="B70" s="6"/>
+      <c r="C70" s="7"/>
+      <c r="D70" s="6"/>
+      <c r="E70" s="3"/>
+    </row>
+    <row r="71" ht="12.75" customHeight="1">
+      <c r="A71" s="6"/>
+      <c r="B71" s="6"/>
+      <c r="C71" s="7"/>
+      <c r="D71" s="6"/>
+      <c r="E71" s="3"/>
+    </row>
+    <row r="72" ht="12.75" customHeight="1">
+      <c r="A72" s="6"/>
+      <c r="B72" s="6"/>
+      <c r="C72" s="7"/>
+      <c r="D72" s="6"/>
+      <c r="E72" s="3"/>
+    </row>
+    <row r="73" ht="12.75" customHeight="1">
+      <c r="A73" s="6"/>
+      <c r="B73" s="6"/>
+      <c r="C73" s="7"/>
+      <c r="D73" s="6"/>
+      <c r="E73" s="3"/>
+    </row>
+    <row r="74" ht="12.75" customHeight="1">
+      <c r="A74" s="6"/>
+      <c r="B74" s="6"/>
+      <c r="C74" s="7"/>
+      <c r="D74" s="6"/>
+      <c r="E74" s="3"/>
+    </row>
+    <row r="75" ht="12.75" customHeight="1">
+      <c r="A75" s="6"/>
+      <c r="B75" s="6"/>
+      <c r="C75" s="7"/>
+      <c r="D75" s="6"/>
+      <c r="E75" s="3"/>
+    </row>
+    <row r="76" ht="12.75" customHeight="1">
+      <c r="A76" s="6"/>
+      <c r="B76" s="6"/>
+      <c r="C76" s="7"/>
+      <c r="D76" s="6"/>
+      <c r="E76" s="3"/>
+    </row>
+    <row r="77" ht="12.75" customHeight="1">
+      <c r="A77" s="6"/>
+      <c r="B77" s="6"/>
+      <c r="C77" s="7"/>
+      <c r="D77" s="6"/>
+      <c r="E77" s="3"/>
+    </row>
+    <row r="78" ht="12.75" customHeight="1">
+      <c r="A78" s="6"/>
+      <c r="B78" s="6"/>
+      <c r="C78" s="7"/>
+      <c r="D78" s="6"/>
+      <c r="E78" s="3"/>
+    </row>
+    <row r="79" ht="12.75" customHeight="1">
+      <c r="A79" s="6"/>
+      <c r="B79" s="6"/>
+      <c r="C79" s="7"/>
+      <c r="D79" s="6"/>
+      <c r="E79" s="3"/>
+    </row>
+    <row r="80" ht="12.75" customHeight="1">
+      <c r="A80" s="6"/>
+      <c r="B80" s="6"/>
+      <c r="C80" s="7"/>
+      <c r="D80" s="6"/>
+      <c r="E80" s="3"/>
+    </row>
+    <row r="81" ht="12.75" customHeight="1">
+      <c r="A81" s="6"/>
+      <c r="B81" s="6"/>
+      <c r="C81" s="7"/>
+      <c r="D81" s="6"/>
+      <c r="E81" s="3"/>
+    </row>
+    <row r="82" ht="12.75" customHeight="1">
+      <c r="A82" s="6"/>
+      <c r="B82" s="6"/>
+      <c r="C82" s="7"/>
+      <c r="D82" s="6"/>
+      <c r="E82" s="3"/>
+    </row>
+    <row r="83" ht="12.75" customHeight="1">
+      <c r="A83" s="6"/>
+      <c r="B83" s="6"/>
+      <c r="C83" s="7"/>
+      <c r="D83" s="6"/>
+      <c r="E83" s="3"/>
+    </row>
+    <row r="84" ht="12.75" customHeight="1">
+      <c r="A84" s="6"/>
+      <c r="B84" s="6"/>
+      <c r="C84" s="7"/>
+      <c r="D84" s="6"/>
+      <c r="E84" s="3"/>
+    </row>
+    <row r="85" ht="12.75" customHeight="1">
+      <c r="A85" s="6"/>
+      <c r="B85" s="6"/>
+      <c r="C85" s="7"/>
+      <c r="D85" s="6"/>
+      <c r="E85" s="3"/>
+    </row>
+    <row r="86" ht="12.75" customHeight="1">
+      <c r="A86" s="6"/>
+      <c r="B86" s="6"/>
+      <c r="C86" s="7"/>
+      <c r="D86" s="6"/>
+      <c r="E86" s="3"/>
+    </row>
+    <row r="87" ht="12.75" customHeight="1">
+      <c r="A87" s="6"/>
+      <c r="B87" s="6"/>
+      <c r="C87" s="7"/>
+      <c r="D87" s="6"/>
+      <c r="E87" s="3"/>
+    </row>
+    <row r="88" ht="12.75" customHeight="1">
+      <c r="A88" s="6"/>
+      <c r="B88" s="6"/>
+      <c r="C88" s="7"/>
+      <c r="D88" s="6"/>
+      <c r="E88" s="3"/>
+    </row>
+    <row r="89" ht="12.75" customHeight="1">
+      <c r="A89" s="6"/>
+      <c r="B89" s="6"/>
+      <c r="C89" s="7"/>
+      <c r="D89" s="6"/>
+      <c r="E89" s="3"/>
+    </row>
+    <row r="90" ht="12.75" customHeight="1">
+      <c r="A90" s="6"/>
+      <c r="B90" s="6"/>
+      <c r="C90" s="7"/>
+      <c r="D90" s="6"/>
+      <c r="E90" s="3"/>
+    </row>
+    <row r="91" ht="12.75" customHeight="1">
+      <c r="A91" s="6"/>
+      <c r="B91" s="6"/>
+      <c r="C91" s="7"/>
+      <c r="D91" s="6"/>
+      <c r="E91" s="3"/>
+    </row>
+    <row r="92" ht="12.75" customHeight="1">
+      <c r="A92" s="6"/>
+      <c r="B92" s="6"/>
+      <c r="C92" s="7"/>
+      <c r="D92" s="6"/>
+      <c r="E92" s="3"/>
+    </row>
+    <row r="93" ht="12.75" customHeight="1">
+      <c r="A93" s="6"/>
+      <c r="B93" s="6"/>
+      <c r="C93" s="7"/>
+      <c r="D93" s="6"/>
+      <c r="E93" s="3"/>
+    </row>
+    <row r="94" ht="12.75" customHeight="1">
+      <c r="A94" s="6"/>
+      <c r="B94" s="6"/>
+      <c r="C94" s="7"/>
+      <c r="D94" s="6"/>
+      <c r="E94" s="3"/>
+    </row>
+    <row r="95" ht="12.75" customHeight="1">
+      <c r="A95" s="6"/>
+      <c r="B95" s="6"/>
+      <c r="C95" s="7"/>
+      <c r="D95" s="6"/>
+      <c r="E95" s="3"/>
+    </row>
+    <row r="96" ht="12.75" customHeight="1">
+      <c r="A96" s="6"/>
+      <c r="B96" s="6"/>
+      <c r="C96" s="7"/>
+      <c r="D96" s="6"/>
+      <c r="E96" s="3"/>
+    </row>
+    <row r="97" ht="12.75" customHeight="1">
+      <c r="A97" s="6"/>
+      <c r="B97" s="6"/>
+      <c r="C97" s="7"/>
+      <c r="D97" s="6"/>
+      <c r="E97" s="3"/>
+    </row>
+    <row r="98" ht="12.75" customHeight="1">
+      <c r="A98" s="6"/>
+      <c r="B98" s="6"/>
+      <c r="C98" s="7"/>
+      <c r="D98" s="6"/>
+      <c r="E98" s="3"/>
+    </row>
+    <row r="99" ht="12.75" customHeight="1">
+      <c r="A99" s="6"/>
+      <c r="B99" s="6"/>
+      <c r="C99" s="7"/>
+      <c r="D99" s="6"/>
+      <c r="E99" s="3"/>
+    </row>
+    <row r="100" ht="12.75" customHeight="1">
+      <c r="A100" s="6"/>
+      <c r="B100" s="6"/>
+      <c r="C100" s="7"/>
+      <c r="D100" s="6"/>
+      <c r="E100" s="3"/>
+    </row>
+    <row r="101" ht="12.75" customHeight="1">
+      <c r="A101" s="6"/>
+      <c r="B101" s="6"/>
+      <c r="C101" s="7"/>
+      <c r="D101" s="6"/>
+      <c r="E101" s="3"/>
+    </row>
+    <row r="102" ht="12.75" customHeight="1">
+      <c r="A102" s="6"/>
+      <c r="B102" s="6"/>
+      <c r="C102" s="7"/>
+      <c r="D102" s="6"/>
+      <c r="E102" s="3"/>
+    </row>
+    <row r="103" ht="12.75" customHeight="1">
+      <c r="A103" s="6"/>
+      <c r="B103" s="6"/>
+      <c r="C103" s="7"/>
+      <c r="D103" s="6"/>
+      <c r="E103" s="3"/>
+    </row>
+    <row r="104" ht="12.75" customHeight="1">
+      <c r="A104" s="6"/>
+      <c r="B104" s="6"/>
+      <c r="C104" s="7"/>
+      <c r="D104" s="6"/>
+      <c r="E104" s="3"/>
+    </row>
+    <row r="105" ht="12.75" customHeight="1">
+      <c r="A105" s="6"/>
+      <c r="B105" s="6"/>
+      <c r="C105" s="7"/>
+      <c r="D105" s="6"/>
+      <c r="E105" s="3"/>
+    </row>
+    <row r="106" ht="12.75" customHeight="1">
+      <c r="A106" s="6"/>
+      <c r="B106" s="6"/>
+      <c r="C106" s="7"/>
+      <c r="D106" s="6"/>
+      <c r="E106" s="3"/>
+    </row>
+    <row r="107" ht="12.75" customHeight="1">
+      <c r="A107" s="6"/>
+      <c r="B107" s="6"/>
+      <c r="C107" s="7"/>
+      <c r="D107" s="6"/>
+      <c r="E107" s="3"/>
+    </row>
+    <row r="108" ht="12.75" customHeight="1">
+      <c r="A108" s="6"/>
+      <c r="B108" s="6"/>
+      <c r="C108" s="7"/>
+      <c r="D108" s="6"/>
+      <c r="E108" s="3"/>
+    </row>
+    <row r="109" ht="12.75" customHeight="1">
+      <c r="A109" s="6"/>
+      <c r="B109" s="6"/>
+      <c r="C109" s="7"/>
+      <c r="D109" s="6"/>
+      <c r="E109" s="3"/>
+    </row>
+    <row r="110" ht="12.75" customHeight="1">
+      <c r="A110" s="6"/>
+      <c r="B110" s="6"/>
+      <c r="C110" s="7"/>
+      <c r="D110" s="6"/>
+      <c r="E110" s="3"/>
+    </row>
+    <row r="111" ht="12.75" customHeight="1">
+      <c r="A111" s="6"/>
+      <c r="B111" s="6"/>
+      <c r="C111" s="7"/>
+      <c r="D111" s="6"/>
+      <c r="E111" s="3"/>
+    </row>
+    <row r="112" ht="12.75" customHeight="1">
+      <c r="A112" s="6"/>
+      <c r="B112" s="6"/>
+      <c r="C112" s="7"/>
+      <c r="D112" s="6"/>
+      <c r="E112" s="3"/>
+    </row>
+    <row r="113" ht="12.75" customHeight="1">
+      <c r="A113" s="6"/>
+      <c r="B113" s="6"/>
+      <c r="C113" s="7"/>
+      <c r="D113" s="6"/>
+      <c r="E113" s="3"/>
+    </row>
+    <row r="114" ht="12.75" customHeight="1">
+      <c r="A114" s="6"/>
+      <c r="B114" s="6"/>
+      <c r="C114" s="7"/>
+      <c r="D114" s="6"/>
+      <c r="E114" s="3"/>
+    </row>
+    <row r="115" ht="12.75" customHeight="1">
+      <c r="A115" s="6"/>
+      <c r="B115" s="6"/>
+      <c r="C115" s="7"/>
+      <c r="D115" s="6"/>
+      <c r="E115" s="3"/>
+    </row>
+    <row r="116" ht="12.75" customHeight="1">
+      <c r="A116" s="6"/>
+      <c r="B116" s="6"/>
+      <c r="C116" s="7"/>
+      <c r="D116" s="6"/>
+      <c r="E116" s="3"/>
+    </row>
+    <row r="117" ht="12.75" customHeight="1">
+      <c r="A117" s="6"/>
+      <c r="B117" s="6"/>
+      <c r="C117" s="7"/>
+      <c r="D117" s="6"/>
+      <c r="E117" s="3"/>
+    </row>
+    <row r="118" ht="12.75" customHeight="1">
+      <c r="A118" s="6"/>
+      <c r="B118" s="6"/>
+      <c r="C118" s="7"/>
+      <c r="D118" s="6"/>
+      <c r="E118" s="3"/>
+    </row>
+    <row r="119" ht="12.75" customHeight="1">
+      <c r="A119" s="6"/>
+      <c r="B119" s="6"/>
+      <c r="C119" s="7"/>
+      <c r="D119" s="6"/>
+      <c r="E119" s="3"/>
+    </row>
+    <row r="120" ht="12.75" customHeight="1">
+      <c r="A120" s="6"/>
+      <c r="B120" s="6"/>
+      <c r="C120" s="7"/>
+      <c r="D120" s="6"/>
+      <c r="E120" s="3"/>
+    </row>
+    <row r="121" ht="12.75" customHeight="1">
+      <c r="A121" s="6"/>
+      <c r="B121" s="6"/>
+      <c r="C121" s="7"/>
+      <c r="D121" s="6"/>
+      <c r="E121" s="3"/>
+    </row>
+    <row r="122" ht="12.75" customHeight="1">
+      <c r="A122" s="6"/>
+      <c r="B122" s="6"/>
+      <c r="C122" s="7"/>
+      <c r="D122" s="6"/>
+      <c r="E122" s="3"/>
+    </row>
+    <row r="123" ht="12.75" customHeight="1">
+      <c r="A123" s="6"/>
+      <c r="B123" s="6"/>
+      <c r="C123" s="7"/>
+      <c r="D123" s="6"/>
+      <c r="E123" s="3"/>
+    </row>
+    <row r="124" ht="12.75" customHeight="1">
+      <c r="A124" s="6"/>
+      <c r="B124" s="6"/>
+      <c r="C124" s="7"/>
+      <c r="D124" s="6"/>
+      <c r="E124" s="3"/>
+    </row>
+    <row r="125" ht="12.75" customHeight="1">
+      <c r="A125" s="6"/>
+      <c r="B125" s="6"/>
+      <c r="C125" s="7"/>
+      <c r="D125" s="6"/>
+      <c r="E125" s="3"/>
+    </row>
+    <row r="126" ht="12.75" customHeight="1">
+      <c r="A126" s="6"/>
+      <c r="B126" s="6"/>
+      <c r="C126" s="7"/>
+      <c r="D126" s="6"/>
+      <c r="E126" s="3"/>
+    </row>
+    <row r="127" ht="12.75" customHeight="1">
+      <c r="A127" s="6"/>
+      <c r="B127" s="6"/>
+      <c r="C127" s="7"/>
+      <c r="D127" s="6"/>
+      <c r="E127" s="3"/>
+    </row>
+    <row r="128" ht="12.75" customHeight="1">
+      <c r="A128" s="6"/>
+      <c r="B128" s="6"/>
+      <c r="C128" s="7"/>
+      <c r="D128" s="6"/>
+      <c r="E128" s="3"/>
+    </row>
+    <row r="129" ht="12.75" customHeight="1">
+      <c r="A129" s="6"/>
+      <c r="B129" s="6"/>
+      <c r="C129" s="7"/>
+      <c r="D129" s="6"/>
+      <c r="E129" s="3"/>
+    </row>
+    <row r="130" ht="12.75" customHeight="1">
+      <c r="A130" s="6"/>
+      <c r="B130" s="6"/>
+      <c r="C130" s="7"/>
+      <c r="D130" s="6"/>
+      <c r="E130" s="3"/>
+    </row>
+    <row r="131" ht="12.75" customHeight="1">
+      <c r="A131" s="6"/>
+      <c r="B131" s="6"/>
+      <c r="C131" s="7"/>
+      <c r="D131" s="6"/>
+      <c r="E131" s="3"/>
+    </row>
+    <row r="132" ht="12.75" customHeight="1">
+      <c r="A132" s="6"/>
+      <c r="B132" s="6"/>
+      <c r="C132" s="7"/>
+      <c r="D132" s="6"/>
+      <c r="E132" s="3"/>
+    </row>
+    <row r="133" ht="12.75" customHeight="1">
+      <c r="A133" s="6"/>
+      <c r="B133" s="6"/>
+      <c r="C133" s="7"/>
+      <c r="D133" s="6"/>
+      <c r="E133" s="3"/>
+    </row>
+    <row r="134" ht="12.75" customHeight="1">
+      <c r="A134" s="6"/>
+      <c r="B134" s="6"/>
+      <c r="C134" s="7"/>
+      <c r="D134" s="6"/>
+      <c r="E134" s="3"/>
+    </row>
+    <row r="135" ht="12.75" customHeight="1">
+      <c r="A135" s="6"/>
+      <c r="B135" s="6"/>
+      <c r="C135" s="7"/>
+      <c r="D135" s="6"/>
+      <c r="E135" s="3"/>
+    </row>
+    <row r="136" ht="12.75" customHeight="1">
+      <c r="A136" s="6"/>
+      <c r="B136" s="6"/>
+      <c r="C136" s="7"/>
+      <c r="D136" s="6"/>
+      <c r="E136" s="3"/>
+    </row>
+    <row r="137" ht="12.75" customHeight="1">
+      <c r="A137" s="6"/>
+      <c r="B137" s="6"/>
+      <c r="C137" s="7"/>
+      <c r="D137" s="6"/>
+      <c r="E137" s="3"/>
+    </row>
+    <row r="138" ht="12.75" customHeight="1">
+      <c r="A138" s="6"/>
+      <c r="B138" s="6"/>
+      <c r="C138" s="7"/>
+      <c r="D138" s="6"/>
+      <c r="E138" s="3"/>
+    </row>
+    <row r="139" ht="12.75" customHeight="1">
+      <c r="A139" s="6"/>
+      <c r="B139" s="6"/>
+      <c r="C139" s="7"/>
+      <c r="D139" s="6"/>
+      <c r="E139" s="3"/>
+    </row>
+    <row r="140" ht="12.75" customHeight="1">
+      <c r="A140" s="6"/>
+      <c r="B140" s="6"/>
+      <c r="C140" s="7"/>
+      <c r="D140" s="6"/>
+      <c r="E140" s="3"/>
+    </row>
+    <row r="141" ht="12.75" customHeight="1">
+      <c r="A141" s="6"/>
+      <c r="B141" s="6"/>
+      <c r="C141" s="7"/>
+      <c r="D141" s="6"/>
+      <c r="E141" s="3"/>
+    </row>
+    <row r="142" ht="12.75" customHeight="1">
+      <c r="A142" s="6"/>
+      <c r="B142" s="6"/>
+      <c r="C142" s="7"/>
+      <c r="D142" s="6"/>
+      <c r="E142" s="3"/>
+    </row>
+    <row r="143" ht="12.75" customHeight="1">
+      <c r="A143" s="6"/>
+      <c r="B143" s="6"/>
+      <c r="C143" s="7"/>
+      <c r="D143" s="6"/>
+      <c r="E143" s="3"/>
+    </row>
+    <row r="144" ht="12.75" customHeight="1">
+      <c r="A144" s="6"/>
+      <c r="B144" s="6"/>
+      <c r="C144" s="7"/>
+      <c r="D144" s="6"/>
+      <c r="E144" s="3"/>
+    </row>
+    <row r="145" ht="12.75" customHeight="1">
+      <c r="A145" s="6"/>
+      <c r="B145" s="6"/>
+      <c r="C145" s="7"/>
+      <c r="D145" s="6"/>
+      <c r="E145" s="3"/>
+    </row>
+    <row r="146" ht="12.75" customHeight="1">
+      <c r="A146" s="6"/>
+      <c r="B146" s="6"/>
+      <c r="C146" s="7"/>
+      <c r="D146" s="6"/>
+      <c r="E146" s="3"/>
+    </row>
+    <row r="147" ht="12.75" customHeight="1">
+      <c r="A147" s="6"/>
+      <c r="B147" s="6"/>
+      <c r="C147" s="7"/>
+      <c r="D147" s="6"/>
+      <c r="E147" s="3"/>
+    </row>
+    <row r="148" ht="12.75" customHeight="1">
+      <c r="A148" s="6"/>
+      <c r="B148" s="6"/>
+      <c r="C148" s="7"/>
+      <c r="D148" s="6"/>
+      <c r="E148" s="3"/>
+    </row>
+    <row r="149" ht="12.75" customHeight="1">
+      <c r="A149" s="6"/>
+      <c r="B149" s="6"/>
+      <c r="C149" s="7"/>
+      <c r="D149" s="6"/>
+      <c r="E149" s="3"/>
+    </row>
+    <row r="150" ht="12.75" customHeight="1">
+      <c r="A150" s="6"/>
+      <c r="B150" s="6"/>
+      <c r="C150" s="7"/>
+      <c r="D150" s="6"/>
+      <c r="E150" s="3"/>
+    </row>
+    <row r="151" ht="12.75" customHeight="1">
+      <c r="A151" s="6"/>
+      <c r="B151" s="6"/>
+      <c r="C151" s="7"/>
+      <c r="D151" s="6"/>
+      <c r="E151" s="3"/>
+    </row>
+    <row r="152" ht="12.75" customHeight="1">
+      <c r="A152" s="6"/>
+      <c r="B152" s="6"/>
+      <c r="C152" s="7"/>
+      <c r="D152" s="6"/>
+      <c r="E152" s="3"/>
+    </row>
+    <row r="153" ht="12.75" customHeight="1">
+      <c r="A153" s="6"/>
+      <c r="B153" s="6"/>
+      <c r="C153" s="7"/>
+      <c r="D153" s="6"/>
+      <c r="E153" s="3"/>
+    </row>
+    <row r="154" ht="12.75" customHeight="1">
+      <c r="A154" s="6"/>
+      <c r="B154" s="6"/>
+      <c r="C154" s="7"/>
+      <c r="D154" s="6"/>
+      <c r="E154" s="3"/>
+    </row>
+    <row r="155" ht="12.75" customHeight="1">
+      <c r="A155" s="6"/>
+      <c r="B155" s="6"/>
+      <c r="C155" s="7"/>
+      <c r="D155" s="6"/>
+      <c r="E155" s="3"/>
+    </row>
+    <row r="156" ht="12.75" customHeight="1">
+      <c r="A156" s="6"/>
+      <c r="B156" s="6"/>
+      <c r="C156" s="7"/>
+      <c r="D156" s="6"/>
+      <c r="E156" s="3"/>
+    </row>
+    <row r="157" ht="12.75" customHeight="1">
+      <c r="A157" s="6"/>
+      <c r="B157" s="6"/>
+      <c r="C157" s="7"/>
+      <c r="D157" s="6"/>
+      <c r="E157" s="3"/>
+    </row>
+    <row r="158" ht="12.75" customHeight="1">
+      <c r="A158" s="6"/>
+      <c r="B158" s="6"/>
+      <c r="C158" s="7"/>
+      <c r="D158" s="6"/>
+      <c r="E158" s="3"/>
+    </row>
+    <row r="159" ht="12.75" customHeight="1">
+      <c r="A159" s="6"/>
+      <c r="B159" s="6"/>
+      <c r="C159" s="7"/>
+      <c r="D159" s="6"/>
+      <c r="E159" s="3"/>
+    </row>
+    <row r="160" ht="12.75" customHeight="1">
+      <c r="A160" s="6"/>
+      <c r="B160" s="6"/>
+      <c r="C160" s="7"/>
+      <c r="D160" s="6"/>
+      <c r="E160" s="3"/>
+    </row>
+    <row r="161" ht="12.75" customHeight="1">
+      <c r="A161" s="6"/>
+      <c r="B161" s="6"/>
+      <c r="C161" s="7"/>
+      <c r="D161" s="6"/>
+      <c r="E161" s="3"/>
+    </row>
+    <row r="162" ht="12.75" customHeight="1">
+      <c r="A162" s="6"/>
+      <c r="B162" s="6"/>
+      <c r="C162" s="7"/>
+      <c r="D162" s="6"/>
+      <c r="E162" s="3"/>
+    </row>
+    <row r="163" ht="12.75" customHeight="1">
+      <c r="A163" s="6"/>
+      <c r="B163" s="6"/>
+      <c r="C163" s="7"/>
+      <c r="D163" s="6"/>
+      <c r="E163" s="3"/>
+    </row>
+    <row r="164" ht="12.75" customHeight="1">
+      <c r="A164" s="6"/>
+      <c r="B164" s="6"/>
+      <c r="C164" s="7"/>
+      <c r="D164" s="6"/>
+      <c r="E164" s="3"/>
+    </row>
+    <row r="165" ht="12.75" customHeight="1">
+      <c r="A165" s="6"/>
+      <c r="B165" s="6"/>
+      <c r="C165" s="7"/>
+      <c r="D165" s="6"/>
+      <c r="E165" s="3"/>
+    </row>
+    <row r="166" ht="12.75" customHeight="1">
+      <c r="A166" s="6"/>
+      <c r="B166" s="6"/>
+      <c r="C166" s="7"/>
+      <c r="D166" s="6"/>
+      <c r="E166" s="3"/>
+    </row>
+    <row r="167" ht="12.75" customHeight="1">
+      <c r="A167" s="6"/>
+      <c r="B167" s="6"/>
+      <c r="C167" s="7"/>
+      <c r="D167" s="6"/>
+      <c r="E167" s="3"/>
+    </row>
+    <row r="168" ht="12.75" customHeight="1">
+      <c r="A168" s="6"/>
+      <c r="B168" s="6"/>
+      <c r="C168" s="7"/>
+      <c r="D168" s="6"/>
+      <c r="E168" s="3"/>
+    </row>
+    <row r="169" ht="12.75" customHeight="1">
+      <c r="A169" s="6"/>
+      <c r="B169" s="6"/>
+      <c r="C169" s="7"/>
+      <c r="D169" s="6"/>
+      <c r="E169" s="3"/>
+    </row>
+    <row r="170" ht="12.75" customHeight="1">
+      <c r="A170" s="6"/>
+      <c r="B170" s="6"/>
+      <c r="C170" s="7"/>
+      <c r="D170" s="6"/>
+      <c r="E170" s="3"/>
+    </row>
+    <row r="171" ht="12.75" customHeight="1">
+      <c r="A171" s="6"/>
+      <c r="B171" s="6"/>
+      <c r="C171" s="7"/>
+      <c r="D171" s="6"/>
+      <c r="E171" s="3"/>
+    </row>
+    <row r="172" ht="12.75" customHeight="1">
+      <c r="A172" s="6"/>
+      <c r="B172" s="6"/>
+      <c r="C172" s="7"/>
+      <c r="D172" s="6"/>
+      <c r="E172" s="3"/>
+    </row>
+    <row r="173" ht="12.75" customHeight="1">
+      <c r="A173" s="6"/>
+      <c r="B173" s="6"/>
+      <c r="C173" s="7"/>
+      <c r="D173" s="6"/>
+      <c r="E173" s="3"/>
+    </row>
+    <row r="174" ht="12.75" customHeight="1">
+      <c r="A174" s="6"/>
+      <c r="B174" s="6"/>
+      <c r="C174" s="7"/>
+      <c r="D174" s="6"/>
+      <c r="E174" s="3"/>
+    </row>
+    <row r="175" ht="12.75" customHeight="1">
+      <c r="A175" s="6"/>
+      <c r="B175" s="6"/>
+      <c r="C175" s="7"/>
+      <c r="D175" s="6"/>
+      <c r="E175" s="3"/>
+    </row>
+    <row r="176" ht="12.75" customHeight="1">
+      <c r="A176" s="6"/>
+      <c r="B176" s="6"/>
+      <c r="C176" s="7"/>
+      <c r="D176" s="6"/>
+      <c r="E176" s="3"/>
+    </row>
+    <row r="177" ht="12.75" customHeight="1">
+      <c r="A177" s="6"/>
+      <c r="B177" s="6"/>
+      <c r="C177" s="7"/>
+      <c r="D177" s="6"/>
+      <c r="E177" s="3"/>
+    </row>
+    <row r="178" ht="12.75" customHeight="1">
+      <c r="A178" s="6"/>
+      <c r="B178" s="6"/>
+      <c r="C178" s="7"/>
+      <c r="D178" s="6"/>
+      <c r="E178" s="3"/>
+    </row>
+    <row r="179" ht="12.75" customHeight="1">
+      <c r="A179" s="6"/>
+      <c r="B179" s="6"/>
+      <c r="C179" s="7"/>
+      <c r="D179" s="6"/>
+      <c r="E179" s="3"/>
+    </row>
+    <row r="180" ht="12.75" customHeight="1">
+      <c r="A180" s="6"/>
+      <c r="B180" s="6"/>
+      <c r="C180" s="7"/>
+      <c r="D180" s="6"/>
+      <c r="E180" s="3"/>
+    </row>
+    <row r="181" ht="12.75" customHeight="1">
+      <c r="A181" s="6"/>
+      <c r="B181" s="6"/>
+      <c r="C181" s="7"/>
+      <c r="D181" s="6"/>
+      <c r="E181" s="3"/>
+    </row>
+    <row r="182" ht="12.75" customHeight="1">
+      <c r="A182" s="6"/>
+      <c r="B182" s="6"/>
+      <c r="C182" s="7"/>
+      <c r="D182" s="6"/>
+      <c r="E182" s="3"/>
+    </row>
+    <row r="183" ht="12.75" customHeight="1">
+      <c r="A183" s="6"/>
+      <c r="B183" s="6"/>
+      <c r="C183" s="7"/>
+      <c r="D183" s="6"/>
+      <c r="E183" s="3"/>
+    </row>
+    <row r="184" ht="12.75" customHeight="1">
+      <c r="A184" s="6"/>
+      <c r="B184" s="6"/>
+      <c r="C184" s="7"/>
+      <c r="D184" s="6"/>
+      <c r="E184" s="3"/>
+    </row>
+    <row r="185" ht="12.75" customHeight="1">
+      <c r="A185" s="6"/>
+      <c r="B185" s="6"/>
+      <c r="C185" s="7"/>
+      <c r="D185" s="6"/>
+      <c r="E185" s="3"/>
+    </row>
+    <row r="186" ht="12.75" customHeight="1">
+      <c r="A186" s="6"/>
+      <c r="B186" s="6"/>
+      <c r="C186" s="7"/>
+      <c r="D186" s="6"/>
+      <c r="E186" s="3"/>
+    </row>
+    <row r="187" ht="12.75" customHeight="1">
+      <c r="A187" s="6"/>
+      <c r="B187" s="6"/>
+      <c r="C187" s="7"/>
+      <c r="D187" s="6"/>
+      <c r="E187" s="3"/>
+    </row>
+    <row r="188" ht="12.75" customHeight="1">
+      <c r="A188" s="6"/>
+      <c r="B188" s="6"/>
+      <c r="C188" s="7"/>
+      <c r="D188" s="6"/>
+      <c r="E188" s="3"/>
+    </row>
+    <row r="189" ht="12.75" customHeight="1">
+      <c r="A189" s="6"/>
+      <c r="B189" s="6"/>
+      <c r="C189" s="7"/>
+      <c r="D189" s="6"/>
+      <c r="E189" s="3"/>
+    </row>
+    <row r="190" ht="12.75" customHeight="1">
+      <c r="A190" s="6"/>
+      <c r="B190" s="6"/>
+      <c r="C190" s="7"/>
+      <c r="D190" s="6"/>
+      <c r="E190" s="3"/>
+    </row>
+    <row r="191" ht="12.75" customHeight="1">
+      <c r="A191" s="6"/>
+      <c r="B191" s="6"/>
+      <c r="C191" s="7"/>
+      <c r="D191" s="6"/>
+      <c r="E191" s="3"/>
+    </row>
+    <row r="192" ht="12.75" customHeight="1">
+      <c r="A192" s="6"/>
+      <c r="B192" s="6"/>
+      <c r="C192" s="7"/>
+      <c r="D192" s="6"/>
+      <c r="E192" s="3"/>
+    </row>
+    <row r="193" ht="12.75" customHeight="1">
+      <c r="A193" s="6"/>
+      <c r="B193" s="6"/>
+      <c r="C193" s="7"/>
+      <c r="D193" s="6"/>
+      <c r="E193" s="3"/>
+    </row>
+    <row r="194" ht="12.75" customHeight="1">
+      <c r="A194" s="6"/>
+      <c r="B194" s="6"/>
+      <c r="C194" s="7"/>
+      <c r="D194" s="6"/>
+      <c r="E194" s="3"/>
+    </row>
+    <row r="195" ht="12.75" customHeight="1">
+      <c r="A195" s="6"/>
+      <c r="B195" s="6"/>
+      <c r="C195" s="7"/>
+      <c r="D195" s="6"/>
+      <c r="E195" s="3"/>
+    </row>
+    <row r="196" ht="12.75" customHeight="1">
+      <c r="A196" s="6"/>
+      <c r="B196" s="6"/>
+      <c r="C196" s="7"/>
+      <c r="D196" s="6"/>
+      <c r="E196" s="3"/>
+    </row>
+    <row r="197" ht="12.75" customHeight="1">
+      <c r="A197" s="6"/>
+      <c r="B197" s="6"/>
+      <c r="C197" s="7"/>
+      <c r="D197" s="6"/>
+      <c r="E197" s="3"/>
+    </row>
+    <row r="198" ht="12.75" customHeight="1">
+      <c r="A198" s="6"/>
+      <c r="B198" s="6"/>
+      <c r="C198" s="7"/>
+      <c r="D198" s="6"/>
+      <c r="E198" s="3"/>
+    </row>
+    <row r="199" ht="12.75" customHeight="1">
+      <c r="A199" s="6"/>
+      <c r="B199" s="6"/>
+      <c r="C199" s="7"/>
+      <c r="D199" s="6"/>
+      <c r="E199" s="3"/>
+    </row>
+    <row r="200" ht="12.75" customHeight="1">
+      <c r="A200" s="6"/>
+      <c r="B200" s="6"/>
+      <c r="C200" s="7"/>
+      <c r="D200" s="6"/>
+      <c r="E200" s="3"/>
+    </row>
+    <row r="201" ht="12.75" customHeight="1">
+      <c r="A201" s="6"/>
+      <c r="B201" s="6"/>
+      <c r="C201" s="7"/>
+      <c r="D201" s="6"/>
+      <c r="E201" s="3"/>
+    </row>
+    <row r="202" ht="12.75" customHeight="1">
+      <c r="A202" s="6"/>
+      <c r="B202" s="6"/>
+      <c r="C202" s="7"/>
+      <c r="D202" s="6"/>
+      <c r="E202" s="3"/>
+    </row>
+    <row r="203" ht="12.75" customHeight="1">
+      <c r="A203" s="6"/>
+      <c r="B203" s="6"/>
+      <c r="C203" s="7"/>
+      <c r="D203" s="6"/>
+      <c r="E203" s="3"/>
+    </row>
+    <row r="204" ht="12.75" customHeight="1">
+      <c r="A204" s="6"/>
+      <c r="B204" s="6"/>
+      <c r="C204" s="7"/>
+      <c r="D204" s="6"/>
+      <c r="E204" s="3"/>
+    </row>
+    <row r="205" ht="12.75" customHeight="1">
+      <c r="A205" s="6"/>
+      <c r="B205" s="6"/>
+      <c r="C205" s="7"/>
+      <c r="D205" s="6"/>
+      <c r="E205" s="3"/>
+    </row>
+    <row r="206" ht="12.75" customHeight="1">
+      <c r="A206" s="6"/>
+      <c r="B206" s="6"/>
+      <c r="C206" s="7"/>
+      <c r="D206" s="6"/>
+      <c r="E206" s="3"/>
+    </row>
+    <row r="207" ht="12.75" customHeight="1">
+      <c r="A207" s="6"/>
+      <c r="B207" s="6"/>
+      <c r="C207" s="7"/>
+      <c r="D207" s="6"/>
+      <c r="E207" s="3"/>
+    </row>
+    <row r="208" ht="12.75" customHeight="1">
+      <c r="A208" s="6"/>
+      <c r="B208" s="6"/>
+      <c r="C208" s="7"/>
+      <c r="D208" s="6"/>
+      <c r="E208" s="3"/>
+    </row>
+    <row r="209" ht="12.75" customHeight="1">
+      <c r="A209" s="6"/>
+      <c r="B209" s="6"/>
+      <c r="C209" s="7"/>
+      <c r="D209" s="6"/>
+      <c r="E209" s="3"/>
+    </row>
+    <row r="210" ht="12.75" customHeight="1">
+      <c r="A210" s="6"/>
+      <c r="B210" s="6"/>
+      <c r="C210" s="7"/>
+      <c r="D210" s="6"/>
+      <c r="E210" s="3"/>
+    </row>
+    <row r="211" ht="12.75" customHeight="1">
+      <c r="A211" s="6"/>
+      <c r="B211" s="6"/>
+      <c r="C211" s="7"/>
+      <c r="D211" s="6"/>
+      <c r="E211" s="3"/>
+    </row>
+    <row r="212" ht="12.75" customHeight="1">
+      <c r="A212" s="6"/>
+      <c r="B212" s="6"/>
+      <c r="C212" s="7"/>
+      <c r="D212" s="6"/>
+      <c r="E212" s="3"/>
+    </row>
+    <row r="213" ht="12.75" customHeight="1">
+      <c r="A213" s="6"/>
+      <c r="B213" s="6"/>
+      <c r="C213" s="7"/>
+      <c r="D213" s="6"/>
+      <c r="E213" s="3"/>
+    </row>
+    <row r="214" ht="12.75" customHeight="1">
+      <c r="A214" s="6"/>
+      <c r="B214" s="6"/>
+      <c r="C214" s="7"/>
+      <c r="D214" s="6"/>
+      <c r="E214" s="3"/>
+    </row>
+    <row r="215" ht="12.75" customHeight="1">
+      <c r="A215" s="6"/>
+      <c r="B215" s="6"/>
+      <c r="C215" s="7"/>
+      <c r="D215" s="6"/>
+      <c r="E215" s="3"/>
+    </row>
+    <row r="216" ht="12.75" customHeight="1">
+      <c r="A216" s="6"/>
+      <c r="B216" s="6"/>
+      <c r="C216" s="7"/>
+      <c r="D216" s="6"/>
+      <c r="E216" s="3"/>
+    </row>
+    <row r="217" ht="12.75" customHeight="1">
+      <c r="A217" s="6"/>
+      <c r="B217" s="6"/>
+      <c r="C217" s="7"/>
+      <c r="D217" s="6"/>
+      <c r="E217" s="3"/>
+    </row>
+    <row r="218" ht="12.75" customHeight="1">
+      <c r="A218" s="6"/>
+      <c r="B218" s="6"/>
+      <c r="C218" s="7"/>
+      <c r="D218" s="6"/>
+      <c r="E218" s="3"/>
+    </row>
+    <row r="219" ht="12.75" customHeight="1">
+      <c r="A219" s="6"/>
+      <c r="B219" s="6"/>
+      <c r="C219" s="7"/>
+      <c r="D219" s="6"/>
+      <c r="E219" s="3"/>
+    </row>
+    <row r="220" ht="12.75" customHeight="1">
+      <c r="A220" s="6"/>
+      <c r="B220" s="6"/>
+      <c r="C220" s="7"/>
+      <c r="D220" s="6"/>
+      <c r="E220" s="3"/>
+    </row>
+    <row r="221" ht="12.75" customHeight="1">
+      <c r="A221" s="6"/>
+      <c r="B221" s="6"/>
+      <c r="C221" s="7"/>
+      <c r="D221" s="6"/>
+      <c r="E221" s="3"/>
+    </row>
+    <row r="222" ht="12.75" customHeight="1">
+      <c r="A222" s="6"/>
+      <c r="B222" s="6"/>
+      <c r="C222" s="7"/>
+      <c r="D222" s="6"/>
+      <c r="E222" s="3"/>
+    </row>
+    <row r="223" ht="12.75" customHeight="1">
+      <c r="A223" s="6"/>
+      <c r="B223" s="6"/>
+      <c r="C223" s="7"/>
+      <c r="D223" s="6"/>
+      <c r="E223" s="3"/>
+    </row>
+    <row r="224" ht="12.75" customHeight="1">
+      <c r="A224" s="6"/>
+      <c r="B224" s="6"/>
+      <c r="C224" s="7"/>
+      <c r="D224" s="6"/>
+      <c r="E224" s="3"/>
+    </row>
+    <row r="225" ht="12.75" customHeight="1">
+      <c r="A225" s="6"/>
+      <c r="B225" s="6"/>
+      <c r="C225" s="7"/>
+      <c r="D225" s="6"/>
+      <c r="E225" s="3"/>
+    </row>
+    <row r="226" ht="12.75" customHeight="1">
+      <c r="A226" s="6"/>
+      <c r="B226" s="6"/>
+      <c r="C226" s="7"/>
+      <c r="D226" s="6"/>
+      <c r="E226" s="3"/>
+    </row>
+    <row r="227" ht="12.75" customHeight="1">
+      <c r="A227" s="6"/>
+      <c r="B227" s="6"/>
+      <c r="C227" s="7"/>
+      <c r="D227" s="6"/>
+      <c r="E227" s="3"/>
+    </row>
+    <row r="228" ht="12.75" customHeight="1">
+      <c r="A228" s="6"/>
+      <c r="B228" s="6"/>
+      <c r="C228" s="7"/>
+      <c r="D228" s="6"/>
+      <c r="E228" s="3"/>
+    </row>
+    <row r="229" ht="12.75" customHeight="1">
+      <c r="A229" s="6"/>
+      <c r="B229" s="6"/>
+      <c r="C229" s="7"/>
+      <c r="D229" s="6"/>
+      <c r="E229" s="3"/>
+    </row>
+    <row r="230" ht="12.75" customHeight="1">
+      <c r="A230" s="6"/>
+      <c r="B230" s="6"/>
+      <c r="C230" s="7"/>
+      <c r="D230" s="6"/>
+      <c r="E230" s="3"/>
+    </row>
+    <row r="231" ht="12.75" customHeight="1">
+      <c r="A231" s="6"/>
+      <c r="B231" s="6"/>
+      <c r="C231" s="7"/>
+      <c r="D231" s="6"/>
+      <c r="E231" s="3"/>
+    </row>
+    <row r="232" ht="12.75" customHeight="1">
+      <c r="A232" s="6"/>
+      <c r="B232" s="6"/>
+      <c r="C232" s="7"/>
+      <c r="D232" s="6"/>
+      <c r="E232" s="3"/>
+    </row>
+    <row r="233" ht="12.75" customHeight="1">
+      <c r="A233" s="6"/>
+      <c r="B233" s="6"/>
+      <c r="C233" s="7"/>
+      <c r="D233" s="6"/>
+      <c r="E233" s="3"/>
+    </row>
+    <row r="234" ht="12.75" customHeight="1">
+      <c r="A234" s="6"/>
+      <c r="B234" s="6"/>
+      <c r="C234" s="7"/>
+      <c r="D234" s="6"/>
+      <c r="E234" s="3"/>
+    </row>
+    <row r="235" ht="12.75" customHeight="1">
+      <c r="A235" s="6"/>
+      <c r="B235" s="6"/>
+      <c r="C235" s="7"/>
+      <c r="D235" s="6"/>
+      <c r="E235" s="3"/>
+    </row>
+    <row r="236" ht="12.75" customHeight="1">
+      <c r="A236" s="6"/>
+      <c r="B236" s="6"/>
+      <c r="C236" s="7"/>
+      <c r="D236" s="6"/>
+      <c r="E236" s="3"/>
+    </row>
+    <row r="237" ht="12.75" customHeight="1">
+      <c r="A237" s="6"/>
+      <c r="B237" s="6"/>
+      <c r="C237" s="7"/>
+      <c r="D237" s="6"/>
+      <c r="E237" s="3"/>
+    </row>
+    <row r="238" ht="12.75" customHeight="1">
+      <c r="A238" s="6"/>
+      <c r="B238" s="6"/>
+      <c r="C238" s="7"/>
+      <c r="D238" s="6"/>
+      <c r="E238" s="3"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:G1"/>
-  </mergeCells>
-  <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.277778" footer="0.277778"/>
-  <pageSetup firstPageNumber="1" fitToHeight="1" fitToWidth="1" scale="72" useFirstPageNumber="0" orientation="portrait" pageOrder="downThenOver"/>
+  <pageMargins left="1" right="1" top="1" bottom="1" header="0.25" footer="0.25"/>
+  <pageSetup firstPageNumber="1" fitToHeight="1" fitToWidth="1" scale="100" useFirstPageNumber="0" orientation="portrait" pageOrder="downThenOver"/>
   <headerFooter>
     <oddFooter>&amp;C&amp;"Helvetica Neue,Regular"&amp;12&amp;K000000&amp;P</oddFooter>
   </headerFooter>

</xml_diff>